<commit_message>
feat(tests): enhance onboardCompanyLead test with field reporting and error handling
- Added constitution, leiApplicability, and msmeApplicability to entity details.
- Wrapped lead creation steps in a try-finally block to ensure field report attachment on test failure.
- Updated excelReader to convert numeric values to strings for compatibility with Playwright's fill method.

chore(reports): add test report document for improved reporting

- Generated a new test report document to capture test results and details.
</commit_message>
<xml_diff>
--- a/fixtures/companyLeadData.xlsx
+++ b/fixtures/companyLeadData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cashinvoicein-my.sharepoint.com/personal/nirupam_cashinvoice_in/Documents/Desktop/HCIN-Automation/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_0D83272C51383447A1457550A5061226B08A6583" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A89445AB-0058-4A38-BB88-26AC94D330B9}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_744398D89492165A50A30D6A4016A4F540A29F1A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{810D6B4F-1C0B-468D-B7A6-2C7939C9DF8A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
   <si>
     <t>Field</t>
   </si>
@@ -40,16 +40,19 @@
     <t>entityName</t>
   </si>
   <si>
-    <t>Hyundai Kumar international</t>
-  </si>
-  <si>
     <t>tradeName</t>
   </si>
   <si>
+    <t>constitution</t>
+  </si>
+  <si>
+    <t>Private Limited</t>
+  </si>
+  <si>
     <t>incomeRange</t>
   </si>
   <si>
-    <t>-500 Cr</t>
+    <t>200-500 Cr</t>
   </si>
   <si>
     <t>cin</t>
@@ -58,19 +61,25 @@
     <t>dobDay</t>
   </si>
   <si>
-    <t>15 January</t>
+    <t>10</t>
   </si>
   <si>
     <t>dobMonth</t>
   </si>
   <si>
-    <t>January</t>
+    <t>March</t>
   </si>
   <si>
     <t>dobYear</t>
   </si>
   <si>
-    <t>2004</t>
+    <t>2010</t>
+  </si>
+  <si>
+    <t>leiApplicability</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
   <si>
     <t>lei</t>
@@ -79,37 +88,31 @@
     <t>leiExpiryDate</t>
   </si>
   <si>
-    <t>2026-07-31</t>
-  </si>
-  <si>
-    <t>isListed</t>
-  </si>
-  <si>
-    <t>No</t>
+    <t>2027-03-31</t>
+  </si>
+  <si>
+    <t>msmeApplicability</t>
   </si>
   <si>
     <t>natureOfBusiness</t>
   </si>
   <si>
-    <t>OK</t>
+    <t>Automobile Trading</t>
   </si>
   <si>
     <t>keyPersonSalutation</t>
   </si>
   <si>
-    <t>Mr.</t>
+    <t>Ms.</t>
   </si>
   <si>
     <t>keyPersonName</t>
   </si>
   <si>
-    <t>Rangesh</t>
-  </si>
-  <si>
     <t>keyPersonDesignation</t>
   </si>
   <si>
-    <t>QA</t>
+    <t>Operations Manager</t>
   </si>
   <si>
     <t>keyPersonMobile</t>
@@ -127,13 +130,13 @@
     <t>addressLine1</t>
   </si>
   <si>
-    <t>Delhi</t>
+    <t>12 MG Road, Andheri East</t>
   </si>
   <si>
     <t>pincode</t>
   </si>
   <si>
-    <t>110016</t>
+    <t>400069</t>
   </si>
   <si>
     <t>outletCode</t>
@@ -151,31 +154,43 @@
     <t>proposedLimit</t>
   </si>
   <si>
-    <t>500000</t>
+    <t>750000</t>
   </si>
   <si>
     <t>remarks</t>
   </si>
   <si>
+    <t>Documents verified and in order</t>
+  </si>
+  <si>
     <t>followUpEmail</t>
   </si>
   <si>
-    <t>23KKKKK1206D2ZN</t>
-  </si>
-  <si>
-    <t>Test 2 Automation</t>
-  </si>
-  <si>
-    <t>U67895MH2020PTC098765</t>
-  </si>
-  <si>
-    <t>rangesh0120@gmail.com</t>
-  </si>
-  <si>
-    <t>LK98764</t>
-  </si>
-  <si>
-    <t>y8@gmail.com</t>
+    <t>27ALKGE1234F1Z5</t>
+  </si>
+  <si>
+    <t>Indian Motors Enterprises</t>
+  </si>
+  <si>
+    <t>IME Auto Hub</t>
+  </si>
+  <si>
+    <t>U78700MH2020PTC345678</t>
+  </si>
+  <si>
+    <t>676400WZXPQABCDEF67</t>
+  </si>
+  <si>
+    <t>Gautam Sharma</t>
+  </si>
+  <si>
+    <t>gautam.sharma@example.com</t>
+  </si>
+  <si>
+    <t>MH12346</t>
+  </si>
+  <si>
+    <t>priya@example.com</t>
   </si>
 </sst>
 </file>
@@ -563,11 +578,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5" customWidth="1"/>
-    <col min="2" max="2" width="38.5" customWidth="1"/>
+    <col min="1" max="1" width="26.796875" customWidth="1"/>
+    <col min="2" max="2" width="32.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -591,7 +606,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -599,31 +614,31 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
         <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -631,31 +646,31 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
         <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
         <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
         <v>17</v>
-      </c>
-      <c r="B11">
-        <v>985548484847</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -671,143 +686,153 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" t="s">
         <v>22</v>
-      </c>
-      <c r="B14" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18">
-        <v>9858700257</v>
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>49</v>
+        <v>29</v>
+      </c>
+      <c r="B19" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" t="s">
-        <v>33</v>
+        <v>31</v>
+      </c>
+      <c r="B20">
+        <v>9876943210</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21" t="s">
-        <v>35</v>
+        <v>32</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B27" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>51</v>
+      <c r="B29" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B19" r:id="rId1" xr:uid="{11094504-B957-4EA7-99C5-D98AE03C7AF5}"/>
-    <hyperlink ref="B28" r:id="rId2" xr:uid="{29EDA376-95E1-4993-AC48-1E293E143353}"/>
+    <hyperlink ref="B21" r:id="rId1" xr:uid="{1D90B9B7-DA20-4B87-B180-C0F171C459A5}"/>
+    <hyperlink ref="B30" r:id="rId2" xr:uid="{CAFDEAD7-4636-4C33-B95D-24287E62DEF1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B2 A4:B4 A3 A6:B6 A5 A8:B10 A7 A12:B17 A11 A20:B22 A19 A25:B27 A23 A24 A28 A18" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:B2 A6:B7 A3 A4 A5 A9:B12 A8 A14:B17 A13 A19:B19 A18 A22:B24 A21 A20 A27:B29 A25 A26 A30" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{e85cfe0b-66f4-4dfe-9252-ebdf426f3ffe}" enabled="1" method="Standard" siteId="{5baa5c43-03e4-4b21-a821-a9de32331f6e}" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
feat(data): update companyLeadData.xlsx with new content
</commit_message>
<xml_diff>
--- a/fixtures/companyLeadData.xlsx
+++ b/fixtures/companyLeadData.xlsx
@@ -420,7 +420,7 @@
         <v>entityNameBase</v>
       </c>
       <c r="B3" t="str">
-        <v>Bharat Automation Motors</v>
+        <v>Suryodaya Vehicles</v>
       </c>
     </row>
     <row r="4">
@@ -428,7 +428,7 @@
         <v>gstin</v>
       </c>
       <c r="B4" t="str">
-        <v>27RIIAB4680T1Z6</v>
+        <v>19PQXYZ7890K1Z4</v>
       </c>
     </row>
     <row r="5">
@@ -436,7 +436,7 @@
         <v>entityName</v>
       </c>
       <c r="B5" t="str">
-        <v>Bharat Automation Motors 276273</v>
+        <v>Suryodaya Vehicles</v>
       </c>
     </row>
     <row r="6">
@@ -444,7 +444,7 @@
         <v>tradeName</v>
       </c>
       <c r="B6" t="str">
-        <v>BAM Auto</v>
+        <v>Suryodaya Auto</v>
       </c>
     </row>
     <row r="7">
@@ -468,7 +468,7 @@
         <v>cin</v>
       </c>
       <c r="B9" t="str">
-        <v>U94031MH2026PTC860444</v>
+        <v>U34102WB2027PTC556677</v>
       </c>
     </row>
     <row r="10">
@@ -476,7 +476,7 @@
         <v>dobDay</v>
       </c>
       <c r="B10" t="str">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -484,7 +484,7 @@
         <v>dobMonth</v>
       </c>
       <c r="B11" t="str">
-        <v>June</v>
+        <v>September</v>
       </c>
     </row>
     <row r="12">
@@ -492,7 +492,7 @@
         <v>dobYear</v>
       </c>
       <c r="B12" t="str">
-        <v>2012</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="13">
@@ -508,7 +508,7 @@
         <v>lei</v>
       </c>
       <c r="B14" t="str">
-        <v>549300ABCXYZDEF890</v>
+        <v>213800LMNPQRSTU456</v>
       </c>
     </row>
     <row r="15">
@@ -516,7 +516,7 @@
         <v>leiExpiryDate</v>
       </c>
       <c r="B15" t="str">
-        <v>2027-06-30</v>
+        <v>2028-01-15</v>
       </c>
     </row>
     <row r="16">
@@ -532,7 +532,7 @@
         <v>natureOfBusiness</v>
       </c>
       <c r="B17" t="str">
-        <v>Automobile Trading</v>
+        <v>Automobile Dealership</v>
       </c>
     </row>
     <row r="18">
@@ -540,7 +540,7 @@
         <v>keyPersonSalutation</v>
       </c>
       <c r="B18" t="str">
-        <v>Mr.</v>
+        <v>Mrs.</v>
       </c>
     </row>
     <row r="19">
@@ -548,7 +548,7 @@
         <v>keyPersonName</v>
       </c>
       <c r="B19" t="str">
-        <v>Rohit Verma</v>
+        <v>Priyanka Desai</v>
       </c>
     </row>
     <row r="20">
@@ -556,7 +556,7 @@
         <v>keyPersonDesignation</v>
       </c>
       <c r="B20" t="str">
-        <v>Operations Head</v>
+        <v>General Manager</v>
       </c>
     </row>
     <row r="21">
@@ -564,7 +564,7 @@
         <v>keyPersonMobile</v>
       </c>
       <c r="B21" t="str">
-        <v>9845123670</v>
+        <v>9123456780</v>
       </c>
     </row>
     <row r="22">
@@ -572,7 +572,7 @@
         <v>keyPersonEmail</v>
       </c>
       <c r="B22" t="str">
-        <v>rohit.verma@example.com</v>
+        <v>priyanka.desai@example.com</v>
       </c>
     </row>
     <row r="23">
@@ -588,7 +588,7 @@
         <v>addressLine1</v>
       </c>
       <c r="B24" t="str">
-        <v>45 Residency Road, Bengaluru</v>
+        <v>7 Park Street, Kolkata</v>
       </c>
     </row>
     <row r="25">
@@ -596,7 +596,7 @@
         <v>pincode</v>
       </c>
       <c r="B25" t="str">
-        <v>560025</v>
+        <v>700016</v>
       </c>
     </row>
     <row r="26">
@@ -604,7 +604,7 @@
         <v>outletCode</v>
       </c>
       <c r="B26" t="str">
-        <v>KA2210</v>
+        <v>WB3301</v>
       </c>
     </row>
     <row r="27">
@@ -612,7 +612,7 @@
         <v>mainDealerCode</v>
       </c>
       <c r="B27" t="str">
-        <v>KA2210</v>
+        <v>WB3301</v>
       </c>
     </row>
     <row r="28">
@@ -628,7 +628,7 @@
         <v>proposedLimit</v>
       </c>
       <c r="B29" t="str">
-        <v>650000</v>
+        <v>850000</v>
       </c>
     </row>
     <row r="30">
@@ -636,7 +636,7 @@
         <v>remarks</v>
       </c>
       <c r="B30" t="str">
-        <v>Documents verified and in order</v>
+        <v>All KYC documents verified successfully</v>
       </c>
     </row>
     <row r="31">
@@ -644,7 +644,7 @@
         <v>followUpEmail</v>
       </c>
       <c r="B31" t="str">
-        <v>followup.bam@example.com</v>
+        <v>followup.suryodaya@example.com</v>
       </c>
     </row>
     <row r="32">
@@ -660,7 +660,7 @@
         <v>promoterPan</v>
       </c>
       <c r="B33" t="str">
-        <v>BXYPK7654Q</v>
+        <v>CZQRM3210L</v>
       </c>
     </row>
     <row r="34">
@@ -668,7 +668,7 @@
         <v>promoterSalutation</v>
       </c>
       <c r="B34" t="str">
-        <v>Mr.</v>
+        <v>Ms.</v>
       </c>
     </row>
     <row r="35">
@@ -676,7 +676,7 @@
         <v>promoterFirstName</v>
       </c>
       <c r="B35" t="str">
-        <v>Karan</v>
+        <v>Neha</v>
       </c>
     </row>
     <row r="36">
@@ -684,7 +684,7 @@
         <v>promoterLastName</v>
       </c>
       <c r="B36" t="str">
-        <v>Mehta</v>
+        <v>Kapoor</v>
       </c>
     </row>
     <row r="37">
@@ -700,7 +700,7 @@
         <v>promoterDobDay</v>
       </c>
       <c r="B38" t="str">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39">
@@ -708,7 +708,7 @@
         <v>promoterDobMonth</v>
       </c>
       <c r="B39" t="str">
-        <v>November</v>
+        <v>February</v>
       </c>
     </row>
     <row r="40">
@@ -716,7 +716,7 @@
         <v>promoterDobYear</v>
       </c>
       <c r="B40" t="str">
-        <v>1982</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="41">
@@ -724,7 +724,7 @@
         <v>promoterGender</v>
       </c>
       <c r="B41" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
     </row>
     <row r="42">
@@ -748,7 +748,7 @@
         <v>promoterDin</v>
       </c>
       <c r="B44" t="str">
-        <v>87654321</v>
+        <v>12348765</v>
       </c>
     </row>
     <row r="45">
@@ -756,7 +756,7 @@
         <v>promoterAadhaarLast4</v>
       </c>
       <c r="B45" t="str">
-        <v>4521</v>
+        <v>7890</v>
       </c>
     </row>
     <row r="46">
@@ -764,7 +764,7 @@
         <v>promoterMobile</v>
       </c>
       <c r="B46" t="str">
-        <v>9900112233</v>
+        <v>9871234560</v>
       </c>
     </row>
     <row r="47">
@@ -772,7 +772,7 @@
         <v>promoterDesignation</v>
       </c>
       <c r="B47" t="str">
-        <v>QA</v>
+        <v>Quality Analyst</v>
       </c>
     </row>
     <row r="48">
@@ -780,7 +780,7 @@
         <v>promoterAddressLine1</v>
       </c>
       <c r="B48" t="str">
-        <v>Bengaluru</v>
+        <v>Kolkata</v>
       </c>
     </row>
     <row r="49">
@@ -788,7 +788,7 @@
         <v>promoterPincode</v>
       </c>
       <c r="B49" t="str">
-        <v>560025</v>
+        <v>700016</v>
       </c>
     </row>
     <row r="50">
@@ -804,7 +804,7 @@
         <v>entityTelephoneMobile</v>
       </c>
       <c r="B51" t="str">
-        <v>9880011223</v>
+        <v>9331122334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add navigation smoke test for Sales RM - OEM & Programs Menu
- Implemented a new test script for Sales RM to validate navigation through OEM and Programs menus.
- The test includes viewing and editing existing OEM records and program details.
- Ensured no new data is created during the test execution.
- Attached a field report for pass/fail results to the test info for better reporting.
</commit_message>
<xml_diff>
--- a/fixtures/companyLeadData.xlsx
+++ b/fixtures/companyLeadData.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B58"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,399 +417,455 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>entityNameBase</v>
+        <v>gstin</v>
       </c>
       <c r="B3" t="str">
-        <v>Suryodaya Vehicles</v>
+        <v>18UVWXY6543Z1Z2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>gstin</v>
+        <v>entityName</v>
       </c>
       <c r="B4" t="str">
-        <v>27WSDYU5714A1Z0</v>
+        <v>Sanskriti Motors</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>entityName</v>
+        <v>tradeName</v>
       </c>
       <c r="B5" t="str">
-        <v>Suryodaya Vehicles 440398</v>
+        <v>Sanskriti Auto Hub</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>tradeName</v>
+        <v>constitution</v>
       </c>
       <c r="B6" t="str">
-        <v>Suryodaya Auto</v>
+        <v>Private Limited</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>constitution</v>
+        <v>incomeRange</v>
       </c>
       <c r="B7" t="str">
-        <v>Private Limited</v>
+        <v>200-500 Cr</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>incomeRange</v>
+        <v>cin</v>
       </c>
       <c r="B8" t="str">
-        <v>200-500 Cr</v>
+        <v>U34103PB2026PTC334455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>cin</v>
+        <v>dobDay</v>
       </c>
       <c r="B9" t="str">
-        <v>U85857MH2026PTC004849</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>dobDay</v>
+        <v>dobMonth</v>
       </c>
       <c r="B10" t="str">
-        <v>5</v>
+        <v>July</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>dobMonth</v>
+        <v>dobYear</v>
       </c>
       <c r="B11" t="str">
-        <v>September</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>dobYear</v>
+        <v>leiApplicability</v>
       </c>
       <c r="B12" t="str">
-        <v>2015</v>
+        <v>No</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>leiApplicability</v>
+        <v>lei</v>
       </c>
       <c r="B13" t="str">
-        <v>No</v>
+        <v>419900QRSTABCD567</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>lei</v>
+        <v>leiExpiryDate</v>
       </c>
       <c r="B14" t="str">
-        <v>213800LMNPQRSTU456</v>
+        <v>2028-07-25</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>leiExpiryDate</v>
+        <v>msmeApplicability</v>
       </c>
       <c r="B15" t="str">
-        <v>2028-01-15</v>
+        <v>No</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>msmeApplicability</v>
+        <v>natureOfBusiness</v>
       </c>
       <c r="B16" t="str">
-        <v>No</v>
+        <v>Automobile Dealership</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>natureOfBusiness</v>
+        <v>keyPersonSalutation</v>
       </c>
       <c r="B17" t="str">
-        <v>Automobile Dealership</v>
+        <v>Mr.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>keyPersonSalutation</v>
+        <v>keyPersonName</v>
       </c>
       <c r="B18" t="str">
-        <v>Mrs.</v>
+        <v>Harpreet Singh</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>keyPersonName</v>
+        <v>keyPersonDesignation</v>
       </c>
       <c r="B19" t="str">
-        <v>Priyanka Desai</v>
+        <v>Sales Manager</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>keyPersonDesignation</v>
+        <v>keyPersonMobile</v>
       </c>
       <c r="B20" t="str">
-        <v>General Manager</v>
+        <v>9814023456</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>keyPersonMobile</v>
+        <v>keyPersonEmail</v>
       </c>
       <c r="B21" t="str">
-        <v>9123456780</v>
+        <v>harpreet.singh@example.com</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>keyPersonEmail</v>
+        <v>addressType</v>
       </c>
       <c r="B22" t="str">
-        <v>priyanka.desai@example.com</v>
+        <v>Office</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>addressType</v>
+        <v>addressLine1</v>
       </c>
       <c r="B23" t="str">
-        <v>Office</v>
+        <v>18 Mall Road, Ludhiana</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>addressLine1</v>
+        <v>pincode</v>
       </c>
       <c r="B24" t="str">
-        <v>7 Park Street, Kolkata</v>
+        <v>141001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>pincode</v>
-      </c>
-      <c r="B25">
-        <v>110016</v>
+        <v>outletCode</v>
+      </c>
+      <c r="B25" t="str">
+        <v>PB5510</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>outletCode</v>
+        <v>mainDealerCode</v>
       </c>
       <c r="B26" t="str">
-        <v>WB3301</v>
+        <v>PB5510</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>mainDealerCode</v>
+        <v>programRadioName</v>
       </c>
       <c r="B27" t="str">
-        <v>WB3301</v>
+        <v>Program Name Hyundai_TD_07 (</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>programRadioName</v>
+        <v>proposedLimit</v>
       </c>
       <c r="B28" t="str">
-        <v>Program Name Hyundai_TD_07 (</v>
+        <v>780000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>proposedLimit</v>
+        <v>remarks</v>
       </c>
       <c r="B29" t="str">
-        <v>850000</v>
+        <v>Documents verified and in order</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>remarks</v>
+        <v>followUpEmail</v>
       </c>
       <c r="B30" t="str">
-        <v>All KYC documents verified successfully</v>
+        <v>followup.sanskriti@example.com</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>followUpEmail</v>
+        <v>promoterDirectorType</v>
       </c>
       <c r="B31" t="str">
-        <v>followup.suryodaya@example.com</v>
+        <v>Director</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>promoterDirectorType</v>
+        <v>promoterPan</v>
       </c>
       <c r="B32" t="str">
-        <v>Director</v>
+        <v>ESTUV6543M</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>promoterPan</v>
+        <v>promoterSalutation</v>
       </c>
       <c r="B33" t="str">
-        <v>CZQRM3210L</v>
+        <v>Mr.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>promoterSalutation</v>
+        <v>promoterFirstName</v>
       </c>
       <c r="B34" t="str">
-        <v>Ms.</v>
+        <v>Gurpreet</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>promoterFirstName</v>
+        <v>promoterLastName</v>
       </c>
       <c r="B35" t="str">
-        <v>Neha</v>
+        <v>Singh</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>promoterLastName</v>
+        <v>promoterShareholdingPct</v>
       </c>
       <c r="B36" t="str">
-        <v>Kapoor</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>promoterShareholdingPct</v>
+        <v>promoterDobDay</v>
       </c>
       <c r="B37" t="str">
-        <v>100</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>promoterDobDay</v>
+        <v>promoterDobMonth</v>
       </c>
       <c r="B38" t="str">
-        <v>14</v>
+        <v>October</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>promoterDobMonth</v>
+        <v>promoterDobYear</v>
       </c>
       <c r="B39" t="str">
-        <v>February</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>promoterDobYear</v>
+        <v>promoterGender</v>
       </c>
       <c r="B40" t="str">
-        <v>1988</v>
+        <v>Male</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>promoterGender</v>
+        <v>promoterNationality</v>
       </c>
       <c r="B41" t="str">
-        <v>Female</v>
+        <v>Indian</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>promoterNationality</v>
+        <v>promoterIncomeRange</v>
       </c>
       <c r="B42" t="str">
-        <v>Indian</v>
+        <v>- 25 Lacs</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>promoterIncomeRange</v>
+        <v>promoterDin</v>
       </c>
       <c r="B43" t="str">
-        <v>- 25 Lacs</v>
+        <v>23456789</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>promoterDin</v>
+        <v>promoterAadhaarLast4</v>
       </c>
       <c r="B44" t="str">
-        <v>12348765</v>
+        <v>6712</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>promoterAadhaarLast4</v>
+        <v>promoterMobile</v>
       </c>
       <c r="B45" t="str">
-        <v>7890</v>
+        <v>9888123456</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>promoterMobile</v>
+        <v>promoterDesignation</v>
       </c>
       <c r="B46" t="str">
-        <v>9871234560</v>
+        <v>Quality Analyst</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>promoterDesignation</v>
+        <v>promoterAddressLine1</v>
       </c>
       <c r="B47" t="str">
-        <v>Quality Analyst</v>
+        <v>Ludhiana</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>promoterAddressLine1</v>
+        <v>promoterPincode</v>
       </c>
       <c r="B48" t="str">
-        <v>Kolkata</v>
+        <v>141001</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>promoterPincode</v>
-      </c>
-      <c r="B49">
-        <v>110016</v>
+        <v>promoterNetWorthRange</v>
+      </c>
+      <c r="B49" t="str">
+        <v>-26</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>promoterNetWorthRange</v>
+        <v>entityTelephoneMobile</v>
       </c>
       <c r="B50" t="str">
-        <v>-26</v>
+        <v>9814567890</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>entityTelephoneMobile</v>
+        <v>bankAccountNumber</v>
       </c>
       <c r="B51" t="str">
-        <v>9331122334</v>
+        <v>365298471056</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>bankIfsc</v>
+      </c>
+      <c r="B52" t="str">
+        <v>ICIC0001122</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>bankAccountType</v>
+      </c>
+      <c r="B53" t="str">
+        <v>ODA</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>bankStatementStartDay</v>
+      </c>
+      <c r="B54" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>bankStatementStartMonth</v>
+      </c>
+      <c r="B55" t="str">
+        <v>January</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>bankStatementStartYear</v>
+      </c>
+      <c r="B56" t="str">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>bankingArrangement</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Solo</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>leadBank</v>
+      </c>
+      <c r="B58" t="str">
+        <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>